<commit_message>
Added experiment with different prompts and updated IRA calculation
</commit_message>
<xml_diff>
--- a/files/unified_pipeline/unified_pipeline/data/results/ira_eval_template.xlsx
+++ b/files/unified_pipeline/unified_pipeline/data/results/ira_eval_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaskca1-my.sharepoint.com/personal/iey738_usask_ca/Documents/Mitacs Summer 2026/documentation-debt-project/files/unified_pipeline/unified_pipeline/data/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_6948E21F603996FC40E56F7638341A976770D61B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DA0EACA-547A-4FD9-91AA-B762803C7871}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_6948E21F603996FC40E56F7638341A976770D61B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7158011E-526D-4A9D-AE5C-89EBC385A560}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="rater_Nasser" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -2205,6 +2206,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2514,6 +2519,11 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="5" width="48" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
     <col min="13" max="13" width="30" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>